<commit_message>
Add validation thresholds to time series validation A few structural optimization
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/AirwayObstruction/AirwayObstruction.xlsx
+++ b/data/human/adult/validation/Scenarios/AirwayObstruction/AirwayObstruction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\human\adult\validation\Scenarios\AirwayObstruction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A08CECF0-5E16-4662-BF42-A676476F2FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D2B48C-73C3-4AB3-A224-94F1BF53BDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30" yWindow="30" windowWidth="28770" windowHeight="17250" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Varied" sheetId="1" r:id="rId1"/>
@@ -369,31 +369,31 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -806,57 +806,57 @@
     <col min="3" max="3" width="15" style="11" customWidth="1"/>
     <col min="4" max="4" width="25" style="11" customWidth="1"/>
     <col min="5" max="5" width="35.5703125" style="11" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" style="11" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" style="11" customWidth="1"/>
     <col min="7" max="7" width="40.42578125" style="11" customWidth="1"/>
     <col min="8" max="8" width="38.5703125" style="11" customWidth="1"/>
     <col min="9" max="16384" width="11.5703125" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="25"/>
+      <c r="D1" s="22"/>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="28.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="26" t="s">
+      <c r="F2" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
       <c r="G3" s="3" t="s">
         <v>9</v>
       </c>
@@ -868,11 +868,11 @@
       <c r="A4" s="12">
         <v>0</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
       <c r="G4" s="4" t="s">
         <v>11</v>
       </c>
@@ -891,50 +891,50 @@
       <c r="D5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25" t="s">
+      <c r="F5" s="22"/>
+      <c r="G5" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="H5" s="25"/>
+      <c r="H5" s="22"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="12"/>
-      <c r="E6" s="27" t="s">
+      <c r="E6" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12"/>
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
-      <c r="E7" s="27" t="s">
+      <c r="E7" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
     </row>
     <row r="8" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
       <c r="G8" s="5" t="s">
         <v>9</v>
       </c>
@@ -946,13 +946,13 @@
       <c r="A9" s="14">
         <v>1</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
       <c r="G9" s="4"/>
       <c r="H9" s="13"/>
     </row>
@@ -960,13 +960,13 @@
       <c r="A10" s="14">
         <v>1</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
       <c r="G10" s="4" t="s">
         <v>22</v>
       </c>
@@ -976,13 +976,13 @@
       <c r="A11" s="14">
         <v>1</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
       <c r="G11" s="4"/>
       <c r="H11" s="13"/>
     </row>
@@ -1028,7 +1028,6 @@
       <c r="E13" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="8"/>
       <c r="G13" s="9"/>
       <c r="H13" s="13"/>
     </row>
@@ -1120,13 +1119,13 @@
       <c r="A18" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
       <c r="G18" s="5" t="s">
         <v>9</v>
       </c>
@@ -1138,13 +1137,13 @@
       <c r="A19" s="14">
         <v>2</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
       <c r="G19" s="4" t="s">
         <v>39</v>
       </c>
@@ -1154,13 +1153,13 @@
       <c r="A20" s="14">
         <v>2</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
       <c r="G20" s="4"/>
       <c r="H20" s="13"/>
     </row>
@@ -1204,7 +1203,7 @@
         <v>55</v>
       </c>
       <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
+      <c r="F22" s="8"/>
       <c r="G22" s="9"/>
       <c r="H22" s="13"/>
     </row>
@@ -1284,13 +1283,13 @@
       <c r="A27" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
       <c r="G27" s="5" t="s">
         <v>41</v>
       </c>
@@ -1302,13 +1301,13 @@
       <c r="A28" s="14">
         <v>3</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
       <c r="G28" s="4" t="s">
         <v>43</v>
       </c>
@@ -1318,13 +1317,13 @@
       <c r="A29" s="14">
         <v>3</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
+      <c r="C29" s="21"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
       <c r="G29" s="4"/>
       <c r="H29" s="13"/>
     </row>
@@ -1462,13 +1461,13 @@
       <c r="A36" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B36" s="20" t="s">
+      <c r="B36" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="21"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
       <c r="G36" s="5" t="s">
         <v>9</v>
       </c>
@@ -1480,13 +1479,13 @@
       <c r="A37" s="14">
         <v>4</v>
       </c>
-      <c r="B37" s="22" t="s">
+      <c r="B37" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C37" s="23"/>
-      <c r="D37" s="23"/>
-      <c r="E37" s="23"/>
-      <c r="F37" s="23"/>
+      <c r="C37" s="21"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
       <c r="G37" s="4" t="s">
         <v>45</v>
       </c>
@@ -1496,13 +1495,13 @@
       <c r="A38" s="14">
         <v>4</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="23"/>
-      <c r="F38" s="23"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="21"/>
       <c r="G38" s="4"/>
       <c r="H38" s="13"/>
     </row>
@@ -1626,13 +1625,13 @@
       <c r="A45" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B45" s="20" t="s">
+      <c r="B45" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C45" s="21"/>
-      <c r="D45" s="21"/>
-      <c r="E45" s="21"/>
-      <c r="F45" s="21"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
       <c r="G45" s="5" t="s">
         <v>9</v>
       </c>
@@ -1644,13 +1643,13 @@
       <c r="A46" s="14">
         <v>5</v>
       </c>
-      <c r="B46" s="22" t="s">
+      <c r="B46" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C46" s="23"/>
-      <c r="D46" s="23"/>
-      <c r="E46" s="23"/>
-      <c r="F46" s="23"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
       <c r="G46" s="4" t="s">
         <v>48</v>
       </c>
@@ -1660,13 +1659,13 @@
       <c r="A47" s="14">
         <v>5</v>
       </c>
-      <c r="B47" s="22" t="s">
+      <c r="B47" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C47" s="23"/>
-      <c r="D47" s="23"/>
-      <c r="E47" s="23"/>
-      <c r="F47" s="23"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
       <c r="G47" s="4"/>
       <c r="H47" s="13"/>
     </row>
@@ -1804,13 +1803,13 @@
       <c r="A54" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B54" s="20" t="s">
+      <c r="B54" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C54" s="21"/>
-      <c r="D54" s="21"/>
-      <c r="E54" s="21"/>
-      <c r="F54" s="21"/>
+      <c r="C54" s="28"/>
+      <c r="D54" s="28"/>
+      <c r="E54" s="28"/>
+      <c r="F54" s="28"/>
       <c r="G54" s="5" t="s">
         <v>9</v>
       </c>
@@ -1822,13 +1821,13 @@
       <c r="A55" s="14">
         <v>6</v>
       </c>
-      <c r="B55" s="22" t="s">
+      <c r="B55" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C55" s="23"/>
-      <c r="D55" s="23"/>
-      <c r="E55" s="23"/>
-      <c r="F55" s="23"/>
+      <c r="C55" s="21"/>
+      <c r="D55" s="21"/>
+      <c r="E55" s="21"/>
+      <c r="F55" s="21"/>
       <c r="G55" s="4" t="s">
         <v>45</v>
       </c>
@@ -1838,13 +1837,13 @@
       <c r="A56" s="14">
         <v>6</v>
       </c>
-      <c r="B56" s="22" t="s">
+      <c r="B56" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="C56" s="23"/>
-      <c r="D56" s="23"/>
-      <c r="E56" s="23"/>
-      <c r="F56" s="23"/>
+      <c r="C56" s="21"/>
+      <c r="D56" s="21"/>
+      <c r="E56" s="21"/>
+      <c r="F56" s="21"/>
       <c r="G56" s="4"/>
       <c r="H56" s="13"/>
     </row>
@@ -1966,6 +1965,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B19:F19"/>
     <mergeCell ref="B55:F55"/>
     <mergeCell ref="B56:F56"/>
     <mergeCell ref="A1:B1"/>
@@ -1982,22 +1997,6 @@
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B54:F54"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B47:F47"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>